<commit_message>
fix: update QC card template — remove surface area row per factory request
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/static/templates/karta_kontroli_jakosci.xlsx
+++ b/app/static/templates/karta_kontroli_jakosci.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Karta kontroli jakości" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Karta kontroli jakości'!$A$1:$I$44</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Karta kontroli jakości'!$A$1:$I$43</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -17,9 +17,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.00\ &quot;m²&quot;"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="13">
     <font>
       <name val="Calibri"/>
@@ -416,18 +414,18 @@
     </border>
     <border>
       <left/>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
         <color auto="1"/>
       </right>
       <top style="thin">
@@ -476,16 +474,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -498,96 +493,93 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -895,152 +887,145 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I44"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="9" customWidth="1" style="1" min="1" max="1"/>
     <col width="10.265625" customWidth="1" style="1" min="2" max="2"/>
     <col width="11.265625" customWidth="1" style="1" min="3" max="3"/>
-    <col width="12" customWidth="1" style="1" min="4" max="4"/>
     <col width="8.53125" customWidth="1" style="1" min="7" max="8"/>
     <col width="8.1328125" customWidth="1" style="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.45" customHeight="1" s="1">
-      <c r="A1" s="37" t="n"/>
-      <c r="B1" s="17" t="n"/>
-      <c r="C1" s="38" t="n"/>
-      <c r="D1" s="34" t="inlineStr">
+      <c r="A1" s="36" t="n"/>
+      <c r="B1" s="30" t="n"/>
+      <c r="C1" s="37" t="n"/>
+      <c r="D1" s="29" t="inlineStr">
         <is>
           <t>DOKUMENT PRODUKCYJNY</t>
         </is>
       </c>
-      <c r="E1" s="17" t="n"/>
-      <c r="F1" s="17" t="n"/>
-      <c r="G1" s="17" t="n"/>
-      <c r="H1" s="17" t="n"/>
-      <c r="I1" s="18" t="n"/>
+      <c r="E1" s="30" t="n"/>
+      <c r="F1" s="30" t="n"/>
+      <c r="G1" s="30" t="n"/>
+      <c r="H1" s="30" t="n"/>
+      <c r="I1" s="31" t="n"/>
     </row>
     <row r="2" ht="33" customHeight="1" s="1">
-      <c r="A2" s="21" t="n"/>
-      <c r="B2" s="19" t="n"/>
+      <c r="A2" s="38" t="n"/>
+      <c r="B2" s="33" t="n"/>
       <c r="C2" s="39" t="n"/>
-      <c r="D2" s="35" t="n"/>
-      <c r="E2" s="19" t="n"/>
-      <c r="F2" s="19" t="n"/>
-      <c r="G2" s="19" t="n"/>
-      <c r="H2" s="19" t="n"/>
-      <c r="I2" s="20" t="n"/>
+      <c r="D2" s="32" t="n"/>
+      <c r="E2" s="33" t="n"/>
+      <c r="F2" s="33" t="n"/>
+      <c r="G2" s="33" t="n"/>
+      <c r="H2" s="33" t="n"/>
+      <c r="I2" s="34" t="n"/>
     </row>
     <row r="3" ht="33" customHeight="1" s="1">
-      <c r="A3" s="29" t="inlineStr">
+      <c r="A3" s="41" t="inlineStr">
         <is>
           <t xml:space="preserve">KARTA KONTROLI JAKOŚCI </t>
         </is>
       </c>
-      <c r="B3" s="11" t="n"/>
-      <c r="C3" s="11" t="n"/>
-      <c r="D3" s="11" t="n"/>
-      <c r="E3" s="11" t="n"/>
-      <c r="F3" s="11" t="n"/>
-      <c r="G3" s="11" t="n"/>
-      <c r="H3" s="11" t="n"/>
-      <c r="I3" s="12" t="n"/>
+      <c r="B3" s="13" t="n"/>
+      <c r="C3" s="13" t="n"/>
+      <c r="D3" s="13" t="n"/>
+      <c r="E3" s="13" t="n"/>
+      <c r="F3" s="13" t="n"/>
+      <c r="G3" s="13" t="n"/>
+      <c r="H3" s="13" t="n"/>
+      <c r="I3" s="15" t="n"/>
     </row>
     <row r="4" ht="41.45" customHeight="1" s="1">
-      <c r="A4" s="42" t="inlineStr">
+      <c r="A4" s="40" t="inlineStr">
         <is>
           <t>ZLECENIE NR (wpisz tutaj numer zlecenia)</t>
         </is>
       </c>
-      <c r="B4" s="11" t="n"/>
-      <c r="C4" s="11" t="n"/>
-      <c r="D4" s="11" t="n"/>
-      <c r="E4" s="11" t="n"/>
-      <c r="F4" s="11" t="n"/>
-      <c r="G4" s="11" t="n"/>
-      <c r="H4" s="11" t="n"/>
-      <c r="I4" s="12" t="n"/>
+      <c r="B4" s="13" t="n"/>
+      <c r="C4" s="13" t="n"/>
+      <c r="D4" s="13" t="n"/>
+      <c r="E4" s="13" t="n"/>
+      <c r="F4" s="13" t="n"/>
+      <c r="G4" s="13" t="n"/>
+      <c r="H4" s="13" t="n"/>
+      <c r="I4" s="15" t="n"/>
     </row>
     <row r="5" ht="36" customHeight="1" s="1">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>KLIENT</t>
         </is>
       </c>
-      <c r="B5" s="11" t="n"/>
-      <c r="C5" s="14" t="n"/>
-      <c r="D5" s="23" t="n"/>
-      <c r="E5" s="11" t="n"/>
-      <c r="F5" s="11" t="n"/>
-      <c r="G5" s="11" t="n"/>
-      <c r="H5" s="11" t="n"/>
-      <c r="I5" s="12" t="n"/>
+      <c r="B5" s="13" t="n"/>
+      <c r="C5" s="11" t="n"/>
+      <c r="D5" s="46" t="n"/>
+      <c r="E5" s="13" t="n"/>
+      <c r="F5" s="13" t="n"/>
+      <c r="G5" s="13" t="n"/>
+      <c r="H5" s="13" t="n"/>
+      <c r="I5" s="15" t="n"/>
     </row>
     <row r="6" ht="48.75" customHeight="1" s="1">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>FARBA</t>
         </is>
       </c>
-      <c r="B6" s="11" t="n"/>
-      <c r="C6" s="14" t="n"/>
-      <c r="D6" s="47" t="n"/>
-      <c r="E6" s="11" t="n"/>
-      <c r="F6" s="11" t="n"/>
-      <c r="G6" s="11" t="n"/>
-      <c r="H6" s="11" t="n"/>
-      <c r="I6" s="12" t="n"/>
+      <c r="B6" s="13" t="n"/>
+      <c r="C6" s="11" t="n"/>
+      <c r="D6" s="17" t="n"/>
+      <c r="E6" s="13" t="n"/>
+      <c r="F6" s="13" t="n"/>
+      <c r="G6" s="13" t="n"/>
+      <c r="H6" s="13" t="n"/>
+      <c r="I6" s="15" t="n"/>
     </row>
     <row r="7" ht="17.35" customHeight="1" s="1">
-      <c r="A7" s="24" t="inlineStr">
+      <c r="A7" s="48" t="inlineStr">
         <is>
           <t xml:space="preserve">Pomiary grubości </t>
         </is>
       </c>
-      <c r="B7" s="11" t="n"/>
-      <c r="C7" s="11" t="n"/>
-      <c r="D7" s="11" t="n"/>
-      <c r="E7" s="11" t="n"/>
-      <c r="F7" s="11" t="n"/>
-      <c r="G7" s="11" t="n"/>
-      <c r="H7" s="11" t="n"/>
-      <c r="I7" s="12" t="n"/>
+      <c r="B7" s="13" t="n"/>
+      <c r="C7" s="13" t="n"/>
+      <c r="D7" s="13" t="n"/>
+      <c r="E7" s="13" t="n"/>
+      <c r="F7" s="13" t="n"/>
+      <c r="G7" s="13" t="n"/>
+      <c r="H7" s="13" t="n"/>
+      <c r="I7" s="15" t="n"/>
     </row>
     <row r="8" ht="15" customHeight="1" s="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Powierzchnia wg standardu ZTP:</t>
+          <t>Ilość sztuk:</t>
         </is>
       </c>
       <c r="B8" s="3" t="n"/>
       <c r="C8" s="3" t="n"/>
-      <c r="D8" s="50" t="n">
-        <v>158.44</v>
-      </c>
+      <c r="D8" s="5" t="n"/>
       <c r="E8" s="3" t="n"/>
       <c r="F8" s="3" t="n"/>
       <c r="G8" s="3" t="n"/>
       <c r="H8" s="3" t="n"/>
-      <c r="I8" s="5" t="n"/>
+      <c r="I8" s="4" t="n"/>
     </row>
     <row r="9" ht="15" customHeight="1" s="1">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Ilość sztuk:</t>
-        </is>
-      </c>
+      <c r="A9" s="6" t="n"/>
       <c r="B9" s="3" t="n"/>
       <c r="C9" s="3" t="n"/>
-      <c r="D9" s="6" t="n"/>
+      <c r="D9" s="3" t="n"/>
       <c r="E9" s="3" t="n"/>
       <c r="F9" s="3" t="n"/>
       <c r="G9" s="3" t="n"/>
       <c r="H9" s="3" t="n"/>
-      <c r="I9" s="5" t="n"/>
+      <c r="I9" s="4" t="n"/>
     </row>
     <row r="10" ht="15" customHeight="1" s="1">
-      <c r="A10" s="7" t="n"/>
+      <c r="A10" s="6" t="n"/>
       <c r="B10" s="3" t="n"/>
       <c r="C10" s="3" t="n"/>
       <c r="D10" s="3" t="n"/>
@@ -1048,10 +1033,10 @@
       <c r="F10" s="3" t="n"/>
       <c r="G10" s="3" t="n"/>
       <c r="H10" s="3" t="n"/>
-      <c r="I10" s="5" t="n"/>
+      <c r="I10" s="4" t="n"/>
     </row>
     <row r="11" ht="15" customHeight="1" s="1">
-      <c r="A11" s="7" t="n"/>
+      <c r="A11" s="6" t="n"/>
       <c r="B11" s="3" t="n"/>
       <c r="C11" s="3" t="n"/>
       <c r="D11" s="3" t="n"/>
@@ -1059,54 +1044,54 @@
       <c r="F11" s="3" t="n"/>
       <c r="G11" s="3" t="n"/>
       <c r="H11" s="3" t="n"/>
-      <c r="I11" s="5" t="n"/>
+      <c r="I11" s="4" t="n"/>
     </row>
     <row r="12" ht="15" customHeight="1" s="1">
-      <c r="A12" s="7" t="n"/>
-      <c r="B12" s="3" t="n"/>
+      <c r="A12" s="24" t="n"/>
+      <c r="B12" s="27" t="n"/>
       <c r="C12" s="3" t="n"/>
-      <c r="D12" s="3" t="n"/>
-      <c r="E12" s="3" t="n"/>
-      <c r="F12" s="3" t="n"/>
-      <c r="G12" s="3" t="n"/>
-      <c r="H12" s="3" t="n"/>
-      <c r="I12" s="5" t="n"/>
+      <c r="D12" s="27" t="n"/>
+      <c r="E12" s="27" t="n"/>
+      <c r="F12" s="27" t="n"/>
+      <c r="G12" s="27" t="n"/>
+      <c r="H12" s="27" t="n"/>
+      <c r="I12" s="4" t="n"/>
     </row>
     <row r="13" ht="15" customHeight="1" s="1">
-      <c r="A13" s="40" t="n"/>
-      <c r="B13" s="41" t="n"/>
+      <c r="A13" s="24" t="n"/>
+      <c r="B13" s="27" t="n"/>
       <c r="C13" s="3" t="n"/>
-      <c r="D13" s="41" t="n"/>
-      <c r="E13" s="41" t="n"/>
-      <c r="F13" s="41" t="n"/>
-      <c r="G13" s="41" t="n"/>
-      <c r="H13" s="41" t="n"/>
-      <c r="I13" s="5" t="n"/>
+      <c r="D13" s="27" t="n"/>
+      <c r="E13" s="27" t="n"/>
+      <c r="F13" s="27" t="n"/>
+      <c r="G13" s="27" t="n"/>
+      <c r="H13" s="27" t="n"/>
+      <c r="I13" s="4" t="n"/>
     </row>
     <row r="14" ht="15" customHeight="1" s="1">
-      <c r="A14" s="40" t="n"/>
-      <c r="B14" s="41" t="n"/>
+      <c r="A14" s="24" t="n"/>
+      <c r="B14" s="27" t="n"/>
       <c r="C14" s="3" t="n"/>
-      <c r="D14" s="41" t="n"/>
-      <c r="E14" s="41" t="n"/>
-      <c r="F14" s="41" t="n"/>
-      <c r="G14" s="41" t="n"/>
-      <c r="H14" s="41" t="n"/>
-      <c r="I14" s="5" t="n"/>
+      <c r="D14" s="27" t="n"/>
+      <c r="E14" s="27" t="n"/>
+      <c r="F14" s="27" t="n"/>
+      <c r="G14" s="27" t="n"/>
+      <c r="H14" s="27" t="n"/>
+      <c r="I14" s="4" t="n"/>
     </row>
     <row r="15" ht="15" customHeight="1" s="1">
-      <c r="A15" s="40" t="n"/>
-      <c r="B15" s="41" t="n"/>
+      <c r="A15" s="6" t="n"/>
+      <c r="B15" s="3" t="n"/>
       <c r="C15" s="3" t="n"/>
-      <c r="D15" s="41" t="n"/>
-      <c r="E15" s="41" t="n"/>
-      <c r="F15" s="41" t="n"/>
-      <c r="G15" s="41" t="n"/>
-      <c r="H15" s="41" t="n"/>
-      <c r="I15" s="5" t="n"/>
+      <c r="D15" s="3" t="n"/>
+      <c r="E15" s="3" t="n"/>
+      <c r="F15" s="3" t="n"/>
+      <c r="G15" s="3" t="n"/>
+      <c r="H15" s="3" t="n"/>
+      <c r="I15" s="4" t="n"/>
     </row>
     <row r="16" ht="15" customHeight="1" s="1">
-      <c r="A16" s="7" t="n"/>
+      <c r="A16" s="6" t="n"/>
       <c r="B16" s="3" t="n"/>
       <c r="C16" s="3" t="n"/>
       <c r="D16" s="3" t="n"/>
@@ -1114,10 +1099,10 @@
       <c r="F16" s="3" t="n"/>
       <c r="G16" s="3" t="n"/>
       <c r="H16" s="3" t="n"/>
-      <c r="I16" s="5" t="n"/>
+      <c r="I16" s="4" t="n"/>
     </row>
     <row r="17" ht="15" customHeight="1" s="1">
-      <c r="A17" s="7" t="n"/>
+      <c r="A17" s="6" t="n"/>
       <c r="B17" s="3" t="n"/>
       <c r="C17" s="3" t="n"/>
       <c r="D17" s="3" t="n"/>
@@ -1125,10 +1110,10 @@
       <c r="F17" s="3" t="n"/>
       <c r="G17" s="3" t="n"/>
       <c r="H17" s="3" t="n"/>
-      <c r="I17" s="5" t="n"/>
+      <c r="I17" s="4" t="n"/>
     </row>
     <row r="18" ht="15" customHeight="1" s="1">
-      <c r="A18" s="7" t="n"/>
+      <c r="A18" s="6" t="n"/>
       <c r="B18" s="3" t="n"/>
       <c r="C18" s="3" t="n"/>
       <c r="D18" s="3" t="n"/>
@@ -1136,76 +1121,76 @@
       <c r="F18" s="3" t="n"/>
       <c r="G18" s="3" t="n"/>
       <c r="H18" s="3" t="n"/>
-      <c r="I18" s="5" t="n"/>
+      <c r="I18" s="4" t="n"/>
     </row>
     <row r="19" ht="15" customHeight="1" s="1">
-      <c r="A19" s="7" t="n"/>
-      <c r="B19" s="3" t="n"/>
+      <c r="A19" s="24" t="n"/>
+      <c r="B19" s="27" t="n"/>
       <c r="C19" s="3" t="n"/>
-      <c r="D19" s="3" t="n"/>
-      <c r="E19" s="3" t="n"/>
-      <c r="F19" s="3" t="n"/>
-      <c r="G19" s="3" t="n"/>
-      <c r="H19" s="3" t="n"/>
-      <c r="I19" s="5" t="n"/>
+      <c r="D19" s="27" t="n"/>
+      <c r="E19" s="27" t="n"/>
+      <c r="F19" s="27" t="n"/>
+      <c r="G19" s="27" t="n"/>
+      <c r="H19" s="27" t="n"/>
+      <c r="I19" s="4" t="n"/>
     </row>
     <row r="20" ht="15" customHeight="1" s="1">
-      <c r="A20" s="40" t="n"/>
-      <c r="B20" s="41" t="n"/>
+      <c r="A20" s="24" t="n"/>
+      <c r="B20" s="27" t="n"/>
       <c r="C20" s="3" t="n"/>
-      <c r="D20" s="41" t="n"/>
-      <c r="E20" s="41" t="n"/>
-      <c r="F20" s="41" t="n"/>
-      <c r="G20" s="41" t="n"/>
-      <c r="H20" s="41" t="n"/>
-      <c r="I20" s="5" t="n"/>
+      <c r="D20" s="27" t="n"/>
+      <c r="E20" s="27" t="n"/>
+      <c r="F20" s="27" t="n"/>
+      <c r="G20" s="27" t="n"/>
+      <c r="H20" s="27" t="n"/>
+      <c r="I20" s="4" t="n"/>
     </row>
     <row r="21" ht="15" customHeight="1" s="1">
-      <c r="A21" s="40" t="n"/>
-      <c r="B21" s="41" t="n"/>
+      <c r="A21" s="24" t="n"/>
+      <c r="B21" s="27" t="n"/>
       <c r="C21" s="3" t="n"/>
-      <c r="D21" s="41" t="n"/>
-      <c r="E21" s="41" t="n"/>
-      <c r="F21" s="41" t="n"/>
-      <c r="G21" s="41" t="n"/>
-      <c r="H21" s="41" t="n"/>
-      <c r="I21" s="5" t="n"/>
+      <c r="D21" s="27" t="n"/>
+      <c r="E21" s="27" t="n"/>
+      <c r="F21" s="27" t="n"/>
+      <c r="G21" s="27" t="n"/>
+      <c r="H21" s="27" t="n"/>
+      <c r="I21" s="4" t="n"/>
     </row>
     <row r="22" ht="15" customHeight="1" s="1">
-      <c r="A22" s="40" t="n"/>
-      <c r="B22" s="41" t="n"/>
+      <c r="A22" s="24" t="n"/>
+      <c r="B22" s="27" t="n"/>
       <c r="C22" s="3" t="n"/>
-      <c r="D22" s="41" t="n"/>
-      <c r="E22" s="41" t="n"/>
-      <c r="F22" s="41" t="n"/>
-      <c r="G22" s="41" t="n"/>
-      <c r="H22" s="41" t="n"/>
-      <c r="I22" s="5" t="n"/>
+      <c r="D22" s="27" t="n"/>
+      <c r="E22" s="27" t="n"/>
+      <c r="F22" s="27" t="n"/>
+      <c r="G22" s="27" t="n"/>
+      <c r="H22" s="27" t="n"/>
+      <c r="I22" s="4" t="n"/>
     </row>
     <row r="23" ht="15" customHeight="1" s="1">
-      <c r="A23" s="40" t="n"/>
-      <c r="B23" s="41" t="n"/>
+      <c r="A23" s="24" t="n"/>
+      <c r="B23" s="27" t="n"/>
       <c r="C23" s="3" t="n"/>
-      <c r="D23" s="41" t="n"/>
-      <c r="E23" s="41" t="n"/>
-      <c r="F23" s="41" t="n"/>
-      <c r="G23" s="41" t="n"/>
-      <c r="H23" s="41" t="n"/>
-      <c r="I23" s="5" t="n"/>
+      <c r="D23" s="27" t="n"/>
+      <c r="E23" s="27" t="n"/>
+      <c r="F23" s="27" t="n"/>
+      <c r="G23" s="27" t="n"/>
+      <c r="H23" s="27" t="n"/>
+      <c r="I23" s="4" t="n"/>
     </row>
     <row r="24" ht="15" customHeight="1" s="1">
-      <c r="A24" s="40" t="n"/>
-      <c r="B24" s="41" t="n"/>
+      <c r="A24" s="6" t="n"/>
+      <c r="B24" s="3" t="n"/>
       <c r="C24" s="3" t="n"/>
-      <c r="D24" s="41" t="n"/>
-      <c r="E24" s="41" t="n"/>
-      <c r="F24" s="41" t="n"/>
-      <c r="G24" s="41" t="n"/>
-      <c r="H24" s="41" t="n"/>
-      <c r="I24" s="5" t="n"/>
+      <c r="D24" s="3" t="n"/>
+      <c r="E24" s="3" t="n"/>
+      <c r="F24" s="3" t="n"/>
+      <c r="G24" s="3" t="n"/>
+      <c r="H24" s="3" t="n"/>
+      <c r="I24" s="4" t="n"/>
     </row>
     <row r="25" ht="15" customHeight="1" s="1">
-      <c r="A25" s="7" t="n"/>
+      <c r="A25" s="6" t="n"/>
       <c r="B25" s="3" t="n"/>
       <c r="C25" s="3" t="n"/>
       <c r="D25" s="3" t="n"/>
@@ -1213,10 +1198,10 @@
       <c r="F25" s="3" t="n"/>
       <c r="G25" s="3" t="n"/>
       <c r="H25" s="3" t="n"/>
-      <c r="I25" s="5" t="n"/>
+      <c r="I25" s="4" t="n"/>
     </row>
     <row r="26" ht="15" customHeight="1" s="1">
-      <c r="A26" s="7" t="n"/>
+      <c r="A26" s="6" t="n"/>
       <c r="B26" s="3" t="n"/>
       <c r="C26" s="3" t="n"/>
       <c r="D26" s="3" t="n"/>
@@ -1224,10 +1209,10 @@
       <c r="F26" s="3" t="n"/>
       <c r="G26" s="3" t="n"/>
       <c r="H26" s="3" t="n"/>
-      <c r="I26" s="5" t="n"/>
+      <c r="I26" s="4" t="n"/>
     </row>
     <row r="27" ht="15" customHeight="1" s="1">
-      <c r="A27" s="7" t="n"/>
+      <c r="A27" s="6" t="n"/>
       <c r="B27" s="3" t="n"/>
       <c r="C27" s="3" t="n"/>
       <c r="D27" s="3" t="n"/>
@@ -1235,10 +1220,10 @@
       <c r="F27" s="3" t="n"/>
       <c r="G27" s="3" t="n"/>
       <c r="H27" s="3" t="n"/>
-      <c r="I27" s="5" t="n"/>
+      <c r="I27" s="4" t="n"/>
     </row>
     <row r="28" ht="15" customHeight="1" s="1">
-      <c r="A28" s="7" t="n"/>
+      <c r="A28" s="6" t="n"/>
       <c r="B28" s="3" t="n"/>
       <c r="C28" s="3" t="n"/>
       <c r="D28" s="3" t="n"/>
@@ -1246,225 +1231,215 @@
       <c r="F28" s="3" t="n"/>
       <c r="G28" s="3" t="n"/>
       <c r="H28" s="3" t="n"/>
-      <c r="I28" s="5" t="n"/>
-    </row>
-    <row r="29" ht="15" customHeight="1" s="1">
-      <c r="A29" s="7" t="n"/>
-      <c r="B29" s="3" t="n"/>
-      <c r="C29" s="3" t="n"/>
-      <c r="D29" s="3" t="n"/>
-      <c r="E29" s="3" t="n"/>
-      <c r="F29" s="3" t="n"/>
-      <c r="G29" s="3" t="n"/>
-      <c r="H29" s="3" t="n"/>
-      <c r="I29" s="5" t="n"/>
-    </row>
-    <row r="30" ht="30.6" customHeight="1" s="1">
-      <c r="A30" s="46" t="inlineStr">
+      <c r="I28" s="4" t="n"/>
+    </row>
+    <row r="29" ht="30.6" customHeight="1" s="1">
+      <c r="A29" s="47" t="inlineStr">
         <is>
           <t>Poprawki</t>
         </is>
       </c>
-      <c r="B30" s="11" t="n"/>
-      <c r="C30" s="11" t="n"/>
-      <c r="D30" s="11" t="n"/>
-      <c r="E30" s="11" t="n"/>
-      <c r="F30" s="11" t="n"/>
-      <c r="G30" s="11" t="n"/>
-      <c r="H30" s="11" t="n"/>
-      <c r="I30" s="12" t="n"/>
-    </row>
-    <row r="31" ht="17.35" customHeight="1" s="1">
-      <c r="A31" s="48" t="inlineStr">
+      <c r="B29" s="13" t="n"/>
+      <c r="C29" s="13" t="n"/>
+      <c r="D29" s="13" t="n"/>
+      <c r="E29" s="13" t="n"/>
+      <c r="F29" s="13" t="n"/>
+      <c r="G29" s="13" t="n"/>
+      <c r="H29" s="13" t="n"/>
+      <c r="I29" s="15" t="n"/>
+    </row>
+    <row r="30" ht="17.35" customHeight="1" s="1">
+      <c r="A30" s="18" t="inlineStr">
         <is>
           <t>Numer profila</t>
         </is>
       </c>
-      <c r="B31" s="14" t="n"/>
-      <c r="C31" s="10" t="inlineStr">
+      <c r="B30" s="11" t="n"/>
+      <c r="C30" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Obwód </t>
         </is>
       </c>
-      <c r="D31" s="32" t="inlineStr">
+      <c r="D30" s="44" t="inlineStr">
         <is>
           <t>Długość</t>
         </is>
       </c>
-      <c r="E31" s="14" t="n"/>
-      <c r="F31" s="32" t="inlineStr">
+      <c r="E30" s="11" t="n"/>
+      <c r="F30" s="44" t="inlineStr">
         <is>
           <t>Ilość</t>
         </is>
       </c>
-      <c r="G31" s="14" t="n"/>
-      <c r="H31" s="31" t="inlineStr">
+      <c r="G30" s="11" t="n"/>
+      <c r="H30" s="43" t="inlineStr">
         <is>
           <t>Rodzaj wady</t>
         </is>
       </c>
-      <c r="I31" s="12" t="n"/>
+      <c r="I30" s="15" t="n"/>
+    </row>
+    <row r="31" ht="15.6" customHeight="1" s="1">
+      <c r="A31" s="20" t="n"/>
+      <c r="B31" s="11" t="n"/>
+      <c r="C31" s="3" t="n"/>
+      <c r="D31" s="16" t="n"/>
+      <c r="E31" s="11" t="n"/>
+      <c r="F31" s="16" t="n"/>
+      <c r="G31" s="11" t="n"/>
+      <c r="H31" s="14" t="n"/>
+      <c r="I31" s="15" t="n"/>
     </row>
     <row r="32" ht="15.6" customHeight="1" s="1">
-      <c r="A32" s="27" t="n"/>
-      <c r="B32" s="14" t="n"/>
+      <c r="A32" s="20" t="n"/>
+      <c r="B32" s="11" t="n"/>
       <c r="C32" s="3" t="n"/>
-      <c r="D32" s="26" t="n"/>
-      <c r="E32" s="14" t="n"/>
-      <c r="F32" s="26" t="n"/>
-      <c r="G32" s="14" t="n"/>
-      <c r="H32" s="25" t="n"/>
-      <c r="I32" s="12" t="n"/>
+      <c r="D32" s="16" t="n"/>
+      <c r="E32" s="11" t="n"/>
+      <c r="F32" s="16" t="n"/>
+      <c r="G32" s="11" t="n"/>
+      <c r="H32" s="14" t="n"/>
+      <c r="I32" s="15" t="n"/>
     </row>
     <row r="33" ht="15.6" customHeight="1" s="1">
-      <c r="A33" s="27" t="n"/>
-      <c r="B33" s="14" t="n"/>
+      <c r="A33" s="20" t="n"/>
+      <c r="B33" s="11" t="n"/>
       <c r="C33" s="3" t="n"/>
-      <c r="D33" s="26" t="n"/>
-      <c r="E33" s="14" t="n"/>
-      <c r="F33" s="26" t="n"/>
-      <c r="G33" s="14" t="n"/>
-      <c r="H33" s="25" t="n"/>
-      <c r="I33" s="12" t="n"/>
+      <c r="D33" s="16" t="n"/>
+      <c r="E33" s="11" t="n"/>
+      <c r="F33" s="16" t="n"/>
+      <c r="G33" s="11" t="n"/>
+      <c r="H33" s="14" t="n"/>
+      <c r="I33" s="15" t="n"/>
     </row>
     <row r="34" ht="15.6" customHeight="1" s="1">
-      <c r="A34" s="27" t="n"/>
-      <c r="B34" s="14" t="n"/>
+      <c r="A34" s="20" t="n"/>
+      <c r="B34" s="11" t="n"/>
       <c r="C34" s="3" t="n"/>
-      <c r="D34" s="26" t="n"/>
-      <c r="E34" s="14" t="n"/>
-      <c r="F34" s="26" t="n"/>
-      <c r="G34" s="14" t="n"/>
-      <c r="H34" s="25" t="n"/>
-      <c r="I34" s="12" t="n"/>
+      <c r="D34" s="16" t="n"/>
+      <c r="E34" s="11" t="n"/>
+      <c r="F34" s="16" t="n"/>
+      <c r="G34" s="11" t="n"/>
+      <c r="H34" s="14" t="n"/>
+      <c r="I34" s="15" t="n"/>
     </row>
     <row r="35" ht="15.6" customHeight="1" s="1">
-      <c r="A35" s="27" t="n"/>
-      <c r="B35" s="14" t="n"/>
+      <c r="A35" s="20" t="n"/>
+      <c r="B35" s="11" t="n"/>
       <c r="C35" s="3" t="n"/>
-      <c r="D35" s="26" t="n"/>
-      <c r="E35" s="14" t="n"/>
-      <c r="F35" s="26" t="n"/>
-      <c r="G35" s="14" t="n"/>
-      <c r="H35" s="25" t="n"/>
-      <c r="I35" s="12" t="n"/>
+      <c r="D35" s="16" t="n"/>
+      <c r="E35" s="11" t="n"/>
+      <c r="F35" s="16" t="n"/>
+      <c r="G35" s="11" t="n"/>
+      <c r="H35" s="14" t="n"/>
+      <c r="I35" s="15" t="n"/>
     </row>
     <row r="36" ht="15.6" customHeight="1" s="1">
-      <c r="A36" s="27" t="n"/>
-      <c r="B36" s="14" t="n"/>
+      <c r="A36" s="20" t="n"/>
+      <c r="B36" s="11" t="n"/>
       <c r="C36" s="3" t="n"/>
-      <c r="D36" s="26" t="n"/>
-      <c r="E36" s="14" t="n"/>
-      <c r="F36" s="26" t="n"/>
-      <c r="G36" s="14" t="n"/>
-      <c r="H36" s="25" t="n"/>
-      <c r="I36" s="12" t="n"/>
+      <c r="D36" s="16" t="n"/>
+      <c r="E36" s="11" t="n"/>
+      <c r="F36" s="16" t="n"/>
+      <c r="G36" s="11" t="n"/>
+      <c r="H36" s="14" t="n"/>
+      <c r="I36" s="15" t="n"/>
     </row>
     <row r="37" ht="15.6" customHeight="1" s="1">
-      <c r="A37" s="27" t="n"/>
-      <c r="B37" s="14" t="n"/>
+      <c r="A37" s="20" t="n"/>
+      <c r="B37" s="11" t="n"/>
       <c r="C37" s="3" t="n"/>
-      <c r="D37" s="26" t="n"/>
-      <c r="E37" s="14" t="n"/>
-      <c r="F37" s="26" t="n"/>
-      <c r="G37" s="14" t="n"/>
-      <c r="H37" s="25" t="n"/>
-      <c r="I37" s="12" t="n"/>
+      <c r="D37" s="16" t="n"/>
+      <c r="E37" s="11" t="n"/>
+      <c r="F37" s="16" t="n"/>
+      <c r="G37" s="11" t="n"/>
+      <c r="H37" s="14" t="n"/>
+      <c r="I37" s="15" t="n"/>
     </row>
     <row r="38" ht="15.6" customHeight="1" s="1">
-      <c r="A38" s="27" t="n"/>
-      <c r="B38" s="14" t="n"/>
+      <c r="A38" s="20" t="n"/>
+      <c r="B38" s="11" t="n"/>
       <c r="C38" s="3" t="n"/>
-      <c r="D38" s="26" t="n"/>
-      <c r="E38" s="14" t="n"/>
-      <c r="F38" s="26" t="n"/>
-      <c r="G38" s="14" t="n"/>
-      <c r="H38" s="25" t="n"/>
-      <c r="I38" s="12" t="n"/>
+      <c r="D38" s="16" t="n"/>
+      <c r="E38" s="11" t="n"/>
+      <c r="F38" s="16" t="n"/>
+      <c r="G38" s="11" t="n"/>
+      <c r="H38" s="14" t="n"/>
+      <c r="I38" s="15" t="n"/>
     </row>
     <row r="39" ht="15.6" customHeight="1" s="1">
-      <c r="A39" s="27" t="n"/>
-      <c r="B39" s="14" t="n"/>
+      <c r="A39" s="10" t="n"/>
+      <c r="B39" s="11" t="n"/>
       <c r="C39" s="3" t="n"/>
-      <c r="D39" s="26" t="n"/>
-      <c r="E39" s="14" t="n"/>
-      <c r="F39" s="26" t="n"/>
-      <c r="G39" s="14" t="n"/>
-      <c r="H39" s="25" t="n"/>
-      <c r="I39" s="12" t="n"/>
-    </row>
-    <row r="40" ht="15.6" customHeight="1" s="1">
-      <c r="A40" s="49" t="n"/>
-      <c r="B40" s="14" t="n"/>
+      <c r="D39" s="42" t="n"/>
+      <c r="E39" s="11" t="n"/>
+      <c r="F39" s="42" t="n"/>
+      <c r="G39" s="11" t="n"/>
+      <c r="H39" s="45" t="n"/>
+      <c r="I39" s="15" t="n"/>
+    </row>
+    <row r="40" ht="14.45" customHeight="1" s="1">
+      <c r="A40" s="24" t="n"/>
+      <c r="B40" s="11" t="n"/>
       <c r="C40" s="3" t="n"/>
-      <c r="D40" s="30" t="n"/>
-      <c r="E40" s="14" t="n"/>
-      <c r="F40" s="30" t="n"/>
-      <c r="G40" s="14" t="n"/>
-      <c r="H40" s="33" t="n"/>
-      <c r="I40" s="12" t="n"/>
-    </row>
-    <row r="41" ht="14.45" customHeight="1" s="1">
-      <c r="A41" s="40" t="n"/>
-      <c r="B41" s="14" t="n"/>
+      <c r="D40" s="27" t="n"/>
+      <c r="E40" s="11" t="n"/>
+      <c r="F40" s="27" t="n"/>
+      <c r="G40" s="11" t="n"/>
+      <c r="H40" s="28" t="n"/>
+      <c r="I40" s="15" t="n"/>
+    </row>
+    <row r="41" ht="15" customHeight="1" s="1">
+      <c r="A41" s="24" t="n"/>
+      <c r="B41" s="11" t="n"/>
       <c r="C41" s="3" t="n"/>
-      <c r="D41" s="41" t="n"/>
-      <c r="E41" s="14" t="n"/>
-      <c r="F41" s="41" t="n"/>
-      <c r="G41" s="14" t="n"/>
+      <c r="D41" s="27" t="n"/>
+      <c r="E41" s="11" t="n"/>
+      <c r="F41" s="27" t="n"/>
+      <c r="G41" s="11" t="n"/>
       <c r="H41" s="28" t="n"/>
-      <c r="I41" s="12" t="n"/>
+      <c r="I41" s="15" t="n"/>
     </row>
     <row r="42" ht="15" customHeight="1" s="1">
-      <c r="A42" s="40" t="n"/>
-      <c r="B42" s="14" t="n"/>
-      <c r="C42" s="3" t="n"/>
-      <c r="D42" s="41" t="n"/>
-      <c r="E42" s="14" t="n"/>
-      <c r="F42" s="41" t="n"/>
-      <c r="G42" s="14" t="n"/>
-      <c r="H42" s="28" t="n"/>
-      <c r="I42" s="12" t="n"/>
-    </row>
-    <row r="43" ht="15" customHeight="1" s="1">
-      <c r="A43" s="43" t="inlineStr">
+      <c r="A42" s="19" t="inlineStr">
         <is>
           <t>Data i godzina zakończenia</t>
         </is>
       </c>
-      <c r="B43" s="11" t="n"/>
-      <c r="C43" s="14" t="n"/>
-      <c r="D43" s="36" t="n"/>
-      <c r="E43" s="11" t="n"/>
-      <c r="F43" s="11" t="n"/>
-      <c r="G43" s="11" t="n"/>
-      <c r="H43" s="11" t="n"/>
-      <c r="I43" s="12" t="n"/>
-    </row>
-    <row r="44" ht="15" customHeight="1" s="1">
-      <c r="A44" s="44" t="inlineStr">
+      <c r="B42" s="13" t="n"/>
+      <c r="C42" s="11" t="n"/>
+      <c r="D42" s="35" t="n"/>
+      <c r="E42" s="13" t="n"/>
+      <c r="F42" s="13" t="n"/>
+      <c r="G42" s="13" t="n"/>
+      <c r="H42" s="13" t="n"/>
+      <c r="I42" s="15" t="n"/>
+    </row>
+    <row r="43" ht="15" customHeight="1" s="1">
+      <c r="A43" s="21" t="inlineStr">
         <is>
           <t>Podpis</t>
         </is>
       </c>
-      <c r="B44" s="15" t="n"/>
-      <c r="C44" s="22" t="n"/>
-      <c r="D44" s="45" t="n"/>
-      <c r="E44" s="15" t="n"/>
-      <c r="F44" s="15" t="n"/>
-      <c r="G44" s="15" t="n"/>
-      <c r="H44" s="15" t="n"/>
-      <c r="I44" s="16" t="n"/>
+      <c r="B43" s="22" t="n"/>
+      <c r="C43" s="23" t="n"/>
+      <c r="D43" s="25" t="n"/>
+      <c r="E43" s="22" t="n"/>
+      <c r="F43" s="22" t="n"/>
+      <c r="G43" s="22" t="n"/>
+      <c r="H43" s="22" t="n"/>
+      <c r="I43" s="26" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="62">
     <mergeCell ref="A7:I7"/>
     <mergeCell ref="H35:I35"/>
+    <mergeCell ref="A30:B30"/>
     <mergeCell ref="H38:I38"/>
     <mergeCell ref="D34:E34"/>
     <mergeCell ref="F34:G34"/>
+    <mergeCell ref="A36:B36"/>
     <mergeCell ref="H41:I41"/>
-    <mergeCell ref="A36:B36"/>
     <mergeCell ref="A3:I3"/>
     <mergeCell ref="D40:E40"/>
     <mergeCell ref="H31:I31"/>
@@ -1472,53 +1447,52 @@
     <mergeCell ref="D31:E31"/>
     <mergeCell ref="F40:G40"/>
     <mergeCell ref="H40:I40"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="H39:I39"/>
+    <mergeCell ref="D1:I2"/>
+    <mergeCell ref="A42:C42"/>
     <mergeCell ref="D43:I43"/>
-    <mergeCell ref="D1:I2"/>
+    <mergeCell ref="F30:G30"/>
     <mergeCell ref="H34:I34"/>
-    <mergeCell ref="H39:I39"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="A1:C2"/>
     <mergeCell ref="A41:B41"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="A37:B37"/>
     <mergeCell ref="F33:G33"/>
-    <mergeCell ref="A37:B37"/>
     <mergeCell ref="D32:E32"/>
     <mergeCell ref="F36:G36"/>
-    <mergeCell ref="F42:G42"/>
+    <mergeCell ref="H36:I36"/>
     <mergeCell ref="F32:G32"/>
-    <mergeCell ref="H36:I36"/>
     <mergeCell ref="D41:E41"/>
+    <mergeCell ref="F41:G41"/>
     <mergeCell ref="A4:I4"/>
     <mergeCell ref="A43:C43"/>
-    <mergeCell ref="F41:G41"/>
     <mergeCell ref="F35:G35"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="A44:C44"/>
+    <mergeCell ref="A29:I29"/>
+    <mergeCell ref="D42:I42"/>
     <mergeCell ref="F38:G38"/>
     <mergeCell ref="H32:I32"/>
     <mergeCell ref="D5:I5"/>
     <mergeCell ref="A33:B33"/>
     <mergeCell ref="D37:E37"/>
-    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="A32:B32"/>
     <mergeCell ref="F31:G31"/>
-    <mergeCell ref="A32:B32"/>
     <mergeCell ref="H37:I37"/>
-    <mergeCell ref="D44:I44"/>
-    <mergeCell ref="A30:I30"/>
     <mergeCell ref="D39:E39"/>
     <mergeCell ref="A35:B35"/>
+    <mergeCell ref="F39:G39"/>
     <mergeCell ref="F37:G37"/>
     <mergeCell ref="A38:B38"/>
-    <mergeCell ref="F39:G39"/>
-    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="D30:E30"/>
     <mergeCell ref="D33:E33"/>
-    <mergeCell ref="H42:I42"/>
     <mergeCell ref="A6:C6"/>
     <mergeCell ref="H33:I33"/>
     <mergeCell ref="D38:E38"/>
     <mergeCell ref="D6:I6"/>
     <mergeCell ref="A31:B31"/>
     <mergeCell ref="A39:B39"/>
-    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="A34:B34"/>
     <mergeCell ref="A40:B40"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.2" footer="0.2"/>

</xml_diff>